<commit_message>
daily reports updated logic
</commit_message>
<xml_diff>
--- a/tmp/dailyReport_Client.xlsx
+++ b/tmp/dailyReport_Client.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82557A2D-63DB-46A6-A00D-A709A120FAFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB36E79-D126-4DFB-BD5B-ABD560384E21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="23">
   <si>
     <t>Contact No:      Email: natco.epcorn@gmail.com / sales@epcorn.com</t>
   </si>
@@ -74,13 +74,25 @@
   </si>
   <si>
     <t>Images</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Regular services Done </t>
+  </si>
+  <si>
+    <t>Total Regular services Missed</t>
+  </si>
+  <si>
+    <t>Total Regular services Pending</t>
+  </si>
+  <si>
+    <t>Total Locations</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,8 +139,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -138,6 +158,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -224,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -266,6 +292,24 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -281,23 +325,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -803,7 +832,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="14.88671875" style="12" customWidth="1"/>
@@ -812,153 +841,169 @@
     <col min="5" max="5" width="38.33203125" style="5" customWidth="1"/>
     <col min="6" max="6" width="31.5546875" style="6" customWidth="1"/>
     <col min="7" max="7" width="16.6640625" style="15" customWidth="1"/>
+    <col min="12" max="12" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="99" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:15" ht="99" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-    </row>
-    <row r="2" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+    </row>
+    <row r="2" spans="1:15" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-    </row>
-    <row r="3" spans="1:7" s="25" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="23" t="s">
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+    </row>
+    <row r="3" spans="1:15" s="20" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="23" t="s">
+      <c r="G3" s="18" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11"/>
       <c r="B4" s="11"/>
       <c r="C4" s="1"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="22"/>
+      <c r="F4" s="17"/>
       <c r="G4" s="14"/>
     </row>
-    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11"/>
       <c r="B5" s="11"/>
       <c r="C5" s="1"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
-      <c r="F5" s="22"/>
+      <c r="F5" s="17"/>
       <c r="G5" s="14"/>
     </row>
-    <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="1"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-      <c r="F6" s="22"/>
+      <c r="F6" s="17"/>
       <c r="G6" s="14"/>
     </row>
-    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
       <c r="C7" s="1"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="22"/>
+      <c r="F7" s="17"/>
       <c r="G7" s="14"/>
-    </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L7" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="M7" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="N7" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="O7" s="28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="1"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="22"/>
+      <c r="F8" s="17"/>
       <c r="G8" s="14"/>
     </row>
-    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11"/>
       <c r="B9" s="11"/>
       <c r="C9" s="1"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="22"/>
+      <c r="F9" s="17"/>
       <c r="G9" s="14"/>
     </row>
-    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11"/>
       <c r="B10" s="11"/>
       <c r="C10" s="1"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="22"/>
+      <c r="F10" s="17"/>
       <c r="G10" s="14"/>
     </row>
-    <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11"/>
       <c r="B11" s="11"/>
       <c r="C11" s="1"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="22"/>
+      <c r="F11" s="17"/>
       <c r="G11" s="14"/>
     </row>
-    <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
       <c r="C12" s="1"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="22"/>
+      <c r="F12" s="17"/>
       <c r="G12" s="14"/>
     </row>
-    <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="1"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
-      <c r="F13" s="22"/>
+      <c r="F13" s="17"/>
       <c r="G13" s="14"/>
     </row>
-    <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="1"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
-      <c r="F14" s="22"/>
+      <c r="F14" s="17"/>
       <c r="G14" s="14"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="G15" s="14"/>
     </row>
   </sheetData>
@@ -988,28 +1033,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="80.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
@@ -1173,28 +1218,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="99" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" s="10" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">

</xml_diff>